<commit_message>
docs: publish authorized assessor source and calibration materials
</commit_message>
<xml_diff>
--- a/references/Tabel Pengisian Nilai (A s.d. E).xlsx
+++ b/references/Tabel Pengisian Nilai (A s.d. E).xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BAWAS_WORKSTATION_Y1\Documents\Mahkamah Agung\Evaluasi AKIP\t-SEMAR\references\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774AE5F5-DABD-45F9-99B7-B21284449CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="27">
   <si>
     <t>Pilihan Jawaban</t>
   </si>
@@ -68,94 +77,234 @@
   </si>
   <si>
     <t>Jika sama sekali tidak ada upaya dalam pemenuhan kriteria penilaian akuntabilitas kinerja.</t>
+  </si>
+  <si>
+    <t>REFERENSI PENILAIAN EVALUASI AKIP</t>
+  </si>
+  <si>
+    <t>A. Keberadaan</t>
+  </si>
+  <si>
+    <t>B. Kualitas</t>
+  </si>
+  <si>
+    <t>Jika kualitas seluruh kriteria telah terpenuhi (100%) dan terdapat upaya inovatif serta layak menjadi percontohan secara nasional.</t>
+  </si>
+  <si>
+    <t>Jika kualitas seluruh kriteria telah terpenuhi (100%) dan terdapat beberapa upaya yang bisa dihargai dari pemenuhan kriteria tersebut.</t>
+  </si>
+  <si>
+    <t>C. Pemanfaatan</t>
+  </si>
+  <si>
+    <t>Catatan</t>
+  </si>
+  <si>
+    <t>Setiap nilai sub-komponen harus dilengkapi keterangan dan bukti dokumen pendukung yang relevan.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="&quot;Google Sans Text&quot;"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF1F1F1F"/>
-      <name val="&quot;Google Sans Text&quot;"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D4E78"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F6FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="5">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1D4E78"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7C9DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7C9DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7C9DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7C9DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7C9DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7C9DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7C9DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFC9A227"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -172,39 +321,52 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Sheet1-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="Sheet1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C9" displayName="Isi_Nilai" name="Isi_Nilai" id="1">
-  <tableColumns count="3">
-    <tableColumn name="Pilihan Jawaban" id="1"/>
-    <tableColumn name="Nilai" id="2"/>
-    <tableColumn name="Penjelasan" id="3"/>
-  </tableColumns>
-  <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
-</table>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -394,123 +556,398 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{AE8601C4-4B73-4459-9093-9ECECCE5D5F9}">
+  <we:reference id="wa200010215" version="2.0.0.1" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010215" version="2.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="bps.codex_control.document_id" value="&quot;5ccbd906-9d69-43ad-8b15-acc2de7066c3&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="17.63"/>
-    <col customWidth="1" min="3" max="3" width="37.63"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="12.7265625" customWidth="1"/>
+    <col min="3" max="3" width="94.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" ht="28" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
+    <row r="4" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2">
-        <v>100.0</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B4" s="9">
+        <v>100</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="2" t="s">
+    <row r="5" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2">
-        <v>90.0</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B5" s="6">
+        <v>90</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2" t="s">
+    <row r="6" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
-        <v>80.0</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B6" s="9">
+        <v>80</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2" t="s">
+    <row r="7" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="2">
-        <v>70.0</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="B7" s="6">
+        <v>70</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2" t="s">
+    <row r="8" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2">
-        <v>60.0</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="B8" s="9">
+        <v>60</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2" t="s">
+    <row r="9" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2">
-        <v>50.0</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="B9" s="6">
+        <v>50</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2" t="s">
+    <row r="10" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2">
-        <v>30.0</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="B10" s="6">
+        <v>30</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2" t="s">
+    <row r="11" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B11" s="6">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>18</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="29" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="9">
+        <v>100</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="29" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="6">
+        <v>90</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="9">
+        <v>80</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="6">
+        <v>70</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B19" s="9">
+        <v>60</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="6">
+        <v>50</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="6">
+        <v>30</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="6">
+        <v>0</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+    </row>
+    <row r="25" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="29" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" s="9">
+        <v>100</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="29" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="6">
+        <v>90</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="9">
+        <v>80</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B29" s="6">
+        <v>70</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="9">
+        <v>60</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" s="6">
+        <v>50</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="6">
+        <v>30</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="12">
+        <v>0</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="14.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C34" s="14"/>
+    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
-  </tableParts>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="B34:C34"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>